<commit_message>
USBD21 relational model update USBD22 create tables and inserts
</commit_message>
<xml_diff>
--- a/sql-scripts/Sprint2/Dataset_Sprint_2_v0a.xlsx
+++ b/sql-scripts/Sprint2/Dataset_Sprint_2_v0a.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rafael\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rafael\IdeaProjects\sem-pi-25-26-g054\sql-scripts\Sprint2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FD82BEC-EFEF-43BA-96A7-6A4A32A8ED13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{261362C4-DC27-4088-B60E-72B5A781F460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" firstSheet="1" activeTab="8" xr2:uid="{7F4AA980-AB96-5943-AE3E-BE2681F30F29}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{7F4AA980-AB96-5943-AE3E-BE2681F30F29}"/>
   </bookViews>
   <sheets>
     <sheet name="Facility" sheetId="1" r:id="rId1"/>
@@ -581,7 +581,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0;[Red]0"/>
-    <numFmt numFmtId="166" formatCode="dd\-mm\-yyyy;@"/>
+    <numFmt numFmtId="165" formatCode="dd\-mm\-yyyy;@"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -641,7 +641,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -676,11 +676,11 @@
       <sheetName val="Wagon"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
       <sheetData sheetId="3"/>
-      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="4"/>
       <sheetData sheetId="5"/>
       <sheetData sheetId="6">
         <row r="8">
@@ -689,7 +689,7 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="7" refreshError="1"/>
+      <sheetData sheetId="7"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -1012,13 +1012,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32AE9BB5-1866-604F-9CDF-A9F9C66D7CCC}">
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:W32"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="18.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1026,7 +1026,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1037,8 +1037,12 @@
         <f>"INSERT INTO StationType (id, description) VALUES (1, 'Freight yards');"</f>
         <v>INSERT INTO StationType (id, description) VALUES (1, 'Freight yards');</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="M2" t="str">
+        <f>"INSERT INTO AreaType (id, name) VALUES (1, 'warehouse');"</f>
+        <v>INSERT INTO AreaType (id, name) VALUES (1, 'warehouse');</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1049,8 +1053,12 @@
         <f>"INSERT INTO StationType (id, description) VALUES (2, 'Stations');"</f>
         <v>INSERT INTO StationType (id, description) VALUES (2, 'Stations');</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="M3" t="str">
+        <f>"INSERT INTO AreaType (id, name) VALUES (2, 'refrigerated area');"</f>
+        <v>INSERT INTO AreaType (id, name) VALUES (2, 'refrigerated area');</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1061,8 +1069,12 @@
         <f>"INSERT INTO StationType (id, description) VALUES (3, 'Terminals');"</f>
         <v>INSERT INTO StationType (id, description) VALUES (3, 'Terminals');</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="M4" t="str">
+        <f>"INSERT INTO AreaType (id, name) VALUES (3, 'grain silo');"</f>
+        <v>INSERT INTO AreaType (id, name) VALUES (3, 'grain silo');</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1070,7 +1082,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1082,7 +1094,7 @@
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (1, 'São Romão',1);</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1090,11 +1102,15 @@
         <v>7</v>
       </c>
       <c r="E7" t="str">
-        <f t="shared" ref="E7:E33" si="0">"INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES ("&amp;A3&amp;", '"&amp;B3&amp;"',1);"</f>
+        <f t="shared" ref="E7:E32" si="0">"INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES ("&amp;A3&amp;", '"&amp;B3&amp;"',1);"</f>
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (2, 'Tamel',1);</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="M7" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,2);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,2);</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1105,8 +1121,12 @@
         <f t="shared" si="0"/>
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (3, 'Senhora das Dores',1);</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="R8" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (2,3);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (2,3);</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1118,7 +1138,7 @@
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (4, 'Lousado',1);</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1129,8 +1149,16 @@
         <f t="shared" si="0"/>
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (5, 'Porto Campanhã',1);</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="M10" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,5);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,5);</v>
+      </c>
+      <c r="R10" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (2,5);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (2,5);</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1141,8 +1169,12 @@
         <f t="shared" si="0"/>
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (6, 'Leandro',1);</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="W11" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (3,6);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (3,6);</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1153,8 +1185,12 @@
         <f t="shared" si="0"/>
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (7, 'Porto São Bento',1);</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="R12" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (2,7);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (2,7);</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1166,7 +1202,7 @@
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (8, 'Barcelos',1);</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1177,8 +1213,12 @@
         <f t="shared" si="0"/>
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (9, 'Vila Nova da Cerveira',1);</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="M14" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,9);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,9);</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1190,7 +1230,7 @@
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (10, 'Midões',1);</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1201,8 +1241,20 @@
         <f t="shared" si="0"/>
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (11, 'Valença',1);</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="M16" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,11);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,11);</v>
+      </c>
+      <c r="R16" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (2,11);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (2,11);</v>
+      </c>
+      <c r="W16" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (3,11);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (3,11);</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1213,8 +1265,12 @@
         <f t="shared" si="0"/>
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (12, 'Darque',1);</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="R17" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (2,12);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (2,12);</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1225,8 +1281,20 @@
         <f t="shared" si="0"/>
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (13, 'Contumil',1);</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="M18" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,13);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,13);</v>
+      </c>
+      <c r="R18" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (2,13);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (2,13);</v>
+      </c>
+      <c r="W18" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (3,13);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (3,13);</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1238,7 +1306,7 @@
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (14, 'Ermesinde',1);</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1250,7 +1318,7 @@
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (15, 'São Frutuoso',1);</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1261,8 +1329,16 @@
         <f t="shared" si="0"/>
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (16, 'São Pedro da Torre',1);</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="M21" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,16);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,16);</v>
+      </c>
+      <c r="R21" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (2,16);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (2,16);</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1273,8 +1349,12 @@
         <f t="shared" si="0"/>
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (17, 'Viana do Castelo',1);</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="M22" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,17);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,17);</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1285,8 +1365,12 @@
         <f t="shared" si="0"/>
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (18, 'Famalicão',1);</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="M23" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,18);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,18);</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1297,8 +1381,12 @@
         <f>"INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES ("&amp;A20&amp;", '"&amp;B20&amp;"',1);"</f>
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (19, 'Barroselas',1);</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="R24" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (2,19);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (2,19);</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A25">
         <v>50</v>
       </c>
@@ -1309,8 +1397,12 @@
         <f t="shared" si="0"/>
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (20, 'Nine',1);</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="W25" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (3,20);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (3,20);</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A26">
         <v>45</v>
       </c>
@@ -1321,8 +1413,16 @@
         <f t="shared" si="0"/>
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (21, 'Caminha',1);</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="M26" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,21);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,21);</v>
+      </c>
+      <c r="R26" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (2,21);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (2,21);</v>
+      </c>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A27">
         <v>48</v>
       </c>
@@ -1334,7 +1434,7 @@
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (22, 'Carvalha',1);</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A28">
         <v>43</v>
       </c>
@@ -1345,29 +1445,69 @@
         <f t="shared" si="0"/>
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (23, 'Carreço',1);</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="W28" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (3,23);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (3,23);</v>
+      </c>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.4">
       <c r="E29" t="str">
         <f t="shared" si="0"/>
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (50, 'Leixões',1);</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="M29" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,50);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,50);</v>
+      </c>
+      <c r="R29" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (2,50);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (2,50);</v>
+      </c>
+      <c r="W29" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (3,50);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (3,50);</v>
+      </c>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.4">
       <c r="E30" t="str">
         <f t="shared" si="0"/>
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (45, 'São Mamede de Infesta',1);</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="M30" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,45);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,45);</v>
+      </c>
+      <c r="R30" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (2,45);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (2,45);</v>
+      </c>
+      <c r="W30" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (3,45);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (3,45);</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.4">
       <c r="E31" t="str">
         <f t="shared" si="0"/>
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (48, 'Leça do Balio',1);</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="M31" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,48);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,48);</v>
+      </c>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.4">
       <c r="E32" t="str">
         <f t="shared" si="0"/>
         <v>INSERT INTO Station (idStation, nameStation, stationTypeId) VALUES (43, 'São Gemil',1);</v>
+      </c>
+      <c r="M32" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,43);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (1,43);</v>
+      </c>
+      <c r="W32" t="str">
+        <f>"INSERT INTO AreaTypeStation (areaId, stationId) VALUES (3,43);"</f>
+        <v>INSERT INTO AreaTypeStation (areaId, stationId) VALUES (3,43);</v>
       </c>
     </row>
   </sheetData>
@@ -3591,7 +3731,7 @@
     </row>
     <row r="27" spans="3:3" x14ac:dyDescent="0.4">
       <c r="C27" t="str">
-        <f t="shared" ref="C27:C35" si="0">"INSERT INTO Locomotive (numberLocomotive, name, yearOfEntry, operationalSpeed, model) VALUES ("&amp;A3&amp;",'"&amp;B3&amp;"',"&amp;E3&amp;","&amp;N3&amp;",1);"</f>
+        <f t="shared" ref="C27:C28" si="0">"INSERT INTO Locomotive (numberLocomotive, name, yearOfEntry, operationalSpeed, model) VALUES ("&amp;A3&amp;",'"&amp;B3&amp;"',"&amp;E3&amp;","&amp;N3&amp;",1);"</f>
         <v>INSERT INTO Locomotive (numberLocomotive, name, yearOfEntry, operationalSpeed, model) VALUES (5623,'Paz',1995,70,1);</v>
       </c>
     </row>
@@ -4256,7 +4396,7 @@
     </row>
     <row r="21" spans="2:2" x14ac:dyDescent="0.4">
       <c r="B21" t="str">
-        <f t="shared" ref="B21:B29" si="1">"INSERT INTO WagonModel (id, nameModel, maker, length, width, height, maxSpeed, payload, volume, bogiesId, wagonsTypeId) VALUES ("&amp;A3&amp;",'"&amp;B3&amp;"','"&amp;C3&amp;"',"&amp;F3&amp;","&amp;G3&amp;","&amp;H3&amp;","&amp;J3&amp;","&amp;K3&amp;","&amp;L3&amp;",5,1);"</f>
+        <f t="shared" ref="B21" si="1">"INSERT INTO WagonModel (id, nameModel, maker, length, width, height, maxSpeed, payload, volume, bogiesId, wagonsTypeId) VALUES ("&amp;A3&amp;",'"&amp;B3&amp;"','"&amp;C3&amp;"',"&amp;F3&amp;","&amp;G3&amp;","&amp;H3&amp;","&amp;J3&amp;","&amp;K3&amp;","&amp;L3&amp;",5,1);"</f>
         <v>INSERT INTO WagonModel (id, nameModel, maker, length, width, height, maxSpeed, payload, volume, bogiesId, wagonsTypeId) VALUES (1278,'Tdgs 41 94 074 1','Equimetal',9640,3120,4165.5,100,26.2,38,5,1);</v>
       </c>
     </row>
@@ -4368,7 +4508,7 @@
         <v>1987</v>
       </c>
       <c r="F3" t="str">
-        <f t="shared" ref="F3:F18" si="0">"INSERT INTO Wagon (numberWagon, weight, yearOfEntry, wagonModelId) VALUES ("&amp;A3&amp;", 21.2,"&amp;D3&amp;",1104);"</f>
+        <f t="shared" ref="F3:F17" si="0">"INSERT INTO Wagon (numberWagon, weight, yearOfEntry, wagonModelId) VALUES ("&amp;A3&amp;", 21.2,"&amp;D3&amp;",1104);"</f>
         <v>INSERT INTO Wagon (numberWagon, weight, yearOfEntry, wagonModelId) VALUES (3563078, 21.2,1987,1104);</v>
       </c>
     </row>
@@ -4926,7 +5066,7 @@
         <v>2005</v>
       </c>
       <c r="F34" t="str">
-        <f t="shared" ref="F34:F44" si="4">"INSERT INTO Wagon (numberWagon, weight, yearOfEntry, wagonModelId) VALUES ("&amp;A34&amp;",24 ,"&amp;D34&amp;",1212);"</f>
+        <f t="shared" ref="F34:F42" si="4">"INSERT INTO Wagon (numberWagon, weight, yearOfEntry, wagonModelId) VALUES ("&amp;A34&amp;",24 ,"&amp;D34&amp;",1212);"</f>
         <v>INSERT INTO Wagon (numberWagon, weight, yearOfEntry, wagonModelId) VALUES (3330002,24 ,2005,1212);</v>
       </c>
     </row>

</xml_diff>

<commit_message>
USBD24 update on anonymous locking with best practices.
</commit_message>
<xml_diff>
--- a/sql-scripts/Sprint2/Dataset_Sprint_2_v0a.xlsx
+++ b/sql-scripts/Sprint2/Dataset_Sprint_2_v0a.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rafael\IdeaProjects\sem-pi-25-26-g054\sql-scripts\Sprint2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{656C7BBF-A9E8-49A5-903C-FDA6A70C0674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{133858DB-BA8D-4F37-B66C-6ADDFDBAB830}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" firstSheet="1" activeTab="8" xr2:uid="{7F4AA980-AB96-5943-AE3E-BE2681F30F29}"/>
+    <workbookView xWindow="-165" yWindow="-165" windowWidth="21930" windowHeight="13110" firstSheet="1" activeTab="9" xr2:uid="{7F4AA980-AB96-5943-AE3E-BE2681F30F29}"/>
   </bookViews>
   <sheets>
     <sheet name="Facility" sheetId="1" r:id="rId1"/>
@@ -2574,7 +2574,7 @@
         <v>2</v>
       </c>
       <c r="K9" t="str">
-        <f t="shared" ref="K9:K29" si="0">"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A3&amp;","&amp;E3&amp;","&amp;F3&amp;",1,"&amp;C3&amp;",'','',3,"&amp;B3&amp;");"</f>
+        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A3&amp;","&amp;E3&amp;","&amp;F3&amp;",1,"&amp;C3&amp;",'','',3,"&amp;B3&amp;");"</f>
         <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (3,8000,2443,1,1,'','',3,2);</v>
       </c>
     </row>
@@ -2601,8 +2601,8 @@
         <v>2</v>
       </c>
       <c r="K10" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (10,8000,26560,1,1,'','',3,3);</v>
+        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A4&amp;","&amp;E4&amp;","&amp;F4&amp;",1,"&amp;C4&amp;",'','',2,"&amp;B4&amp;");"</f>
+        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (10,8000,26560,1,1,'','',2,3);</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.4">
@@ -2628,8 +2628,8 @@
         <v>2</v>
       </c>
       <c r="K11" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (11,8000,10000,1,2,'','',3,3);</v>
+        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A5&amp;","&amp;E5&amp;","&amp;F5&amp;",1,"&amp;C5&amp;",'','',2,"&amp;B5&amp;");"</f>
+        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (11,8000,10000,1,2,'','',2,3);</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.4">
@@ -2655,8 +2655,8 @@
         <v>1</v>
       </c>
       <c r="K12" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (15,8000,5286,1,1,'','',3,4);</v>
+        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A6&amp;","&amp;E6&amp;","&amp;F6&amp;",1,"&amp;C6&amp;",'','',2,"&amp;B6&amp;");"</f>
+        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (15,8000,5286,1,1,'','',2,4);</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.4">
@@ -2688,8 +2688,8 @@
         <v>864</v>
       </c>
       <c r="K13" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (16,8000,6000,1,2,'','',3,4);</v>
+        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A7&amp;","&amp;E7&amp;","&amp;F7&amp;",1,"&amp;C7&amp;",'','',2,"&amp;B7&amp;");"</f>
+        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (16,8000,6000,1,2,'','',2,4);</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.4">
@@ -2715,8 +2715,8 @@
         <v>1</v>
       </c>
       <c r="K14" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (14,8000,10387,1,1,'','',3,5);</v>
+        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A8&amp;","&amp;E8&amp;","&amp;F8&amp;",1,"&amp;C8&amp;",'','',2,"&amp;B8&amp;");"</f>
+        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (14,8000,10387,1,1,'','',2,5);</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.4">
@@ -2748,8 +2748,8 @@
         <v>266</v>
       </c>
       <c r="K15" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (12,8000,12000,1,2,'','',3,5);</v>
+        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A9&amp;","&amp;E9&amp;","&amp;F9&amp;",1,"&amp;C9&amp;",'','',2,"&amp;B9&amp;");"</f>
+        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (12,8000,12000,1,2,'','',2,5);</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.4">
@@ -2775,8 +2775,8 @@
         <v>1</v>
       </c>
       <c r="K16" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (13,8000,3100,1,3,'','',3,5);</v>
+        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A10&amp;","&amp;E10&amp;","&amp;F10&amp;",1,"&amp;C10&amp;",'','',2,"&amp;B10&amp;");"</f>
+        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (13,8000,3100,1,3,'','',2,5);</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.4">
@@ -2802,8 +2802,8 @@
         <v>2</v>
       </c>
       <c r="K17" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (20,6400,4890,1,1,'','',3,6);</v>
+        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A11&amp;","&amp;E11&amp;","&amp;F11&amp;",1,"&amp;C11&amp;",'','',2,"&amp;B11&amp;");"</f>
+        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (20,6400,4890,1,1,'','',2,6);</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.4">
@@ -2829,8 +2829,8 @@
         <v>2</v>
       </c>
       <c r="K18" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (18,8000,6000,1,1,'','',3,7);</v>
+        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A12&amp;","&amp;E12&amp;","&amp;F12&amp;",1,"&amp;C12&amp;",'','',1,"&amp;B12&amp;");"</f>
+        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (18,8000,6000,1,1,'','',1,7);</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.4">
@@ -2856,8 +2856,8 @@
         <v>2</v>
       </c>
       <c r="K19" t="str">
-        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A13&amp;","&amp;E13&amp;","&amp;F13&amp;",1,"&amp;C13&amp;","&amp;H13&amp;","&amp;I13&amp;",3,"&amp;B13&amp;");"</f>
-        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (21,8000,5000,1,2,2000,864,3,7);</v>
+        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A13&amp;","&amp;E13&amp;","&amp;F13&amp;",1,"&amp;C13&amp;","&amp;H13&amp;","&amp;I13&amp;",1,"&amp;B13&amp;");"</f>
+        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (21,8000,5000,1,2,2000,864,1,7);</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.4">
@@ -2883,8 +2883,8 @@
         <v>2</v>
       </c>
       <c r="K20" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (22,8000,12000,1,3,'','',3,7);</v>
+        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A14&amp;","&amp;E14&amp;","&amp;F14&amp;",1,"&amp;C14&amp;",'','',1,"&amp;B14&amp;");"</f>
+        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (22,8000,12000,1,3,'','',1,7);</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.4">
@@ -2910,8 +2910,8 @@
         <v>2</v>
       </c>
       <c r="K21" t="str">
-        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A15&amp;","&amp;E15&amp;","&amp;F15&amp;",1,"&amp;C15&amp;","&amp;H15&amp;","&amp;I15&amp;",3,"&amp;B15&amp;");"</f>
-        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (25,8000,20829,1,1,11000,266,3,8);</v>
+        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A15&amp;","&amp;E15&amp;","&amp;F15&amp;",1,"&amp;C15&amp;","&amp;H15&amp;","&amp;I15&amp;",1,"&amp;B15&amp;");"</f>
+        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (25,8000,20829,1,1,11000,266,1,8);</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.4">
@@ -2937,8 +2937,8 @@
         <v>2</v>
       </c>
       <c r="K22" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (26,8000,4264,1,1,'','',3,9);</v>
+        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A16&amp;","&amp;E16&amp;","&amp;F16&amp;",1,"&amp;C16&amp;",'','',1,"&amp;B16&amp;");"</f>
+        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (26,8000,4264,1,1,'','',1,9);</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.4">
@@ -2964,48 +2964,49 @@
         <v>2</v>
       </c>
       <c r="K23" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (30,8000,3883,1,1,'','',3,21);</v>
+        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A17&amp;","&amp;E17&amp;","&amp;F17&amp;",1,"&amp;C17&amp;",'','',2,"&amp;B17&amp;");"</f>
+        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (30,8000,3883,1,1,'','',2,21);</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.4">
       <c r="K24" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (31,8400,1174,1,1,'','',3,22);</v>
+        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A18&amp;","&amp;E18&amp;","&amp;F18&amp;",1,"&amp;C18&amp;",'','',2,"&amp;B18&amp;");"</f>
+        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (31,8400,1174,1,1,'','',2,22);</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.4">
       <c r="K25" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (32,8000,2534,1,2,'','',3,22);</v>
+        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A19&amp;","&amp;E19&amp;","&amp;F19&amp;",1,"&amp;C19&amp;",'','',2,"&amp;B19&amp;");"</f>
+        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (32,8000,2534,1,2,'','',2,22);</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.4">
       <c r="K26" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (33,8000,1566,1,1,'','',3,23);</v>
+        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A20&amp;","&amp;E20&amp;","&amp;F20&amp;",1,"&amp;C20&amp;",'','',2,"&amp;B20&amp;");"</f>
+        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (33,8000,1566,1,1,'','',2,23);</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.4">
       <c r="K27" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (34,8000,1453,1,2,'','',3,23);</v>
+        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A21&amp;","&amp;E21&amp;","&amp;F21&amp;",1,"&amp;C21&amp;",'','',2,"&amp;B21&amp;");"</f>
+        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (34,8000,1453,1,2,'','',2,23);</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.4">
       <c r="K28" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (35,8100,3597,1,1,'','',3,24);</v>
+        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A22&amp;","&amp;E22&amp;","&amp;F22&amp;",1,"&amp;C22&amp;",'','',2,"&amp;B22&amp;");"</f>
+        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (35,8100,3597,1,1,'','',2,24);</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.4">
       <c r="K29" t="str">
-        <f t="shared" si="0"/>
-        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (36,8000,4334,1,2,'','',3,24);</v>
+        <f>"INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES ("&amp;A23&amp;","&amp;E23&amp;","&amp;F23&amp;",1,"&amp;C23&amp;",'','',2,"&amp;B23&amp;");"</f>
+        <v>INSERT INTO LineSegment (id, maximumWeigh, lenght, isElectrified, segmentOrder, sidingPosition, sidingLength, lineSegmentsTypeid, lineId) VALUES (36,8000,4334,1,2,'','',2,24);</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>